<commit_message>
Allow optional notes & optional case in Excel import; enable editing of unpaid expenses
</commit_message>
<xml_diff>
--- a/assets/templates/expense_template.xlsx
+++ b/assets/templates/expense_template.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="23">
   <si>
     <t xml:space="preserve">Date</t>
   </si>
@@ -22,15 +22,15 @@
     <t xml:space="preserve">Category</t>
   </si>
   <si>
+    <t xml:space="preserve">Compensated</t>
+  </si>
+  <si>
     <t xml:space="preserve">Case</t>
   </si>
   <si>
     <t xml:space="preserve">Court</t>
   </si>
   <si>
-    <t xml:space="preserve">Compensated</t>
-  </si>
-  <si>
     <t xml:space="preserve">Notes</t>
   </si>
   <si>
@@ -40,15 +40,15 @@
     <t xml:space="preserve">Court Fees</t>
   </si>
   <si>
+    <t xml:space="preserve">No</t>
+  </si>
+  <si>
     <t xml:space="preserve">State v. Sharma</t>
   </si>
   <si>
     <t xml:space="preserve">High Court of Delhi</t>
   </si>
   <si>
-    <t xml:space="preserve">No</t>
-  </si>
-  <si>
     <t xml:space="preserve">Certified copy urgent fee</t>
   </si>
   <si>
@@ -58,15 +58,15 @@
     <t xml:space="preserve">Travel &amp; Transport</t>
   </si>
   <si>
+    <t xml:space="preserve">Yes</t>
+  </si>
+  <si>
     <t xml:space="preserve">Mehta v. Union of India</t>
   </si>
   <si>
     <t xml:space="preserve">Supreme Court of India</t>
   </si>
   <si>
-    <t xml:space="preserve">Yes</t>
-  </si>
-  <si>
     <t xml:space="preserve">Cab to Court 2</t>
   </si>
   <si>
@@ -76,7 +76,10 @@
     <t xml:space="preserve">Printing &amp; Stationery</t>
   </si>
   <si>
-    <t xml:space="preserve">Paperbook printouts 60 pages</t>
+    <t xml:space="preserve">General</t>
+  </si>
+  <si>
+    <t xml:space="preserve"/>
   </si>
 </sst>
 </file>
@@ -413,13 +416,13 @@
         <v>9</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
   </sheetData>

</xml_diff>